<commit_message>
Regenerate DP4 Excel tables for 10 13C resonances
Co-authored-by: mehmetalagoz <mehmetalagoz@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/dp4_oxime/DP4_Sarotti_ZoneB_1H_tam.xlsx
+++ b/dp4_oxime/DP4_Sarotti_ZoneB_1H_tam.xlsx
@@ -457,7 +457,7 @@
         <v>15</v>
       </c>
       <c r="F2">
-        <v>29.92796666666666</v>
+        <v>29.927967</v>
       </c>
       <c r="G2" t="s">
         <v>15</v>
@@ -480,7 +480,7 @@
         <v>16</v>
       </c>
       <c r="F3">
-        <v>27.75243333333333</v>
+        <v>27.752433</v>
       </c>
       <c r="G3" t="s">
         <v>22</v>

</xml_diff>